<commit_message>
Launch ledger: record both launched sets as deployed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJUn53DicDcqHAh1hw7jdv
</commit_message>
<xml_diff>
--- a/deliverables/coolinens-launch/bulk/COOLINENS_Launch_Ledger_20261004.xlsx
+++ b/deliverables/coolinens-launch/bulk/COOLINENS_Launch_Ledger_20261004.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), bulk upload</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
@@ -1899,17 +1899,17 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P16" s="3" t="inlineStr">
@@ -1997,17 +1997,17 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S17" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P18" s="3" t="inlineStr">
@@ -2193,17 +2193,17 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S18" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P19" s="3" t="inlineStr">
@@ -2291,17 +2291,17 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S19" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P20" s="3" t="inlineStr">
@@ -2389,17 +2389,17 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
@@ -2487,17 +2487,17 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P22" s="3" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S22" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr">
@@ -2683,17 +2683,17 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S23" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
@@ -2781,17 +2781,17 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S25" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T25" s="2" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>deployed</t>
         </is>
       </c>
       <c r="P26" s="3" t="inlineStr">
@@ -2977,17 +2977,17 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>Zarlish (PPC), prepared</t>
+          <t>Zarlish (PPC)</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr">
@@ -8141,12 +8141,12 @@
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N80" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N80" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8205,12 +8205,12 @@
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N81" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N81" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8269,12 +8269,12 @@
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N82" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N82" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8333,12 +8333,12 @@
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N83" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N83" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8401,12 +8401,12 @@
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N84" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N84" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8465,12 +8465,12 @@
       </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N85" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N85" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8525,12 +8525,12 @@
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N86" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N86" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8589,12 +8589,12 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N87" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N87" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8653,12 +8653,12 @@
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N88" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N88" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8717,12 +8717,12 @@
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N89" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8785,12 +8785,12 @@
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N90" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N90" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8849,12 +8849,12 @@
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N91" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N91" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8909,12 +8909,12 @@
       </c>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N92" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N92" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -8973,12 +8973,12 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N93" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N93" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9037,12 +9037,12 @@
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N94" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N94" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9101,12 +9101,12 @@
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N95" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N95" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9169,12 +9169,12 @@
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N96" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N96" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9229,12 +9229,12 @@
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N97" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9293,12 +9293,12 @@
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N98" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N98" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9357,12 +9357,12 @@
       </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N99" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N99" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9421,12 +9421,12 @@
       </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N100" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N100" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9489,12 +9489,12 @@
       </c>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N101" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N101" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9549,12 +9549,12 @@
       </c>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N102" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9613,12 +9613,12 @@
       </c>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N103" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9677,12 +9677,12 @@
       </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N104" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9741,12 +9741,12 @@
       </c>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N105" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9809,12 +9809,12 @@
       </c>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N106" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N106" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9873,12 +9873,12 @@
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N107" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9933,12 +9933,12 @@
       </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N108" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -9997,12 +9997,12 @@
       </c>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N109" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10061,12 +10061,12 @@
       </c>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N110" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N110" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10125,12 +10125,12 @@
       </c>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N111" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N111" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10193,12 +10193,12 @@
       </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N112" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10257,12 +10257,12 @@
       </c>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N113" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10317,12 +10317,12 @@
       </c>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N114" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10381,12 +10381,12 @@
       </c>
       <c r="M115" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N115" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N115" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10445,12 +10445,12 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N116" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N116" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10509,12 +10509,12 @@
       </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N117" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N117" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10577,12 +10577,12 @@
       </c>
       <c r="M118" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N118" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N118" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10641,12 +10641,12 @@
       </c>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N119" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N119" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10701,12 +10701,12 @@
       </c>
       <c r="M120" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N120" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N120" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10765,12 +10765,12 @@
       </c>
       <c r="M121" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N121" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N121" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10829,12 +10829,12 @@
       </c>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N122" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N122" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10893,12 +10893,12 @@
       </c>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N123" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N123" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -10961,12 +10961,12 @@
       </c>
       <c r="M124" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N124" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N124" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11025,12 +11025,12 @@
       </c>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N125" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N125" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11085,12 +11085,12 @@
       </c>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N126" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N126" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11149,12 +11149,12 @@
       </c>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N127" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N127" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11213,12 +11213,12 @@
       </c>
       <c r="M128" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N128" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N128" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11277,12 +11277,12 @@
       </c>
       <c r="M129" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N129" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N129" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11345,12 +11345,12 @@
       </c>
       <c r="M130" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N130" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N130" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11409,12 +11409,12 @@
       </c>
       <c r="M131" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N131" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N131" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11469,12 +11469,12 @@
       </c>
       <c r="M132" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N132" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N132" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11533,12 +11533,12 @@
       </c>
       <c r="M133" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N133" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N133" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11597,12 +11597,12 @@
       </c>
       <c r="M134" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N134" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N134" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11661,12 +11661,12 @@
       </c>
       <c r="M135" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N135" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N135" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11729,12 +11729,12 @@
       </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N136" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N136" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11793,12 +11793,12 @@
       </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N137" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N137" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11853,12 +11853,12 @@
       </c>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N138" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N138" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11917,12 +11917,12 @@
       </c>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N139" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N139" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -11981,12 +11981,12 @@
       </c>
       <c r="M140" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N140" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N140" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12045,12 +12045,12 @@
       </c>
       <c r="M141" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N141" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N141" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12113,12 +12113,12 @@
       </c>
       <c r="M142" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N142" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N142" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12177,12 +12177,12 @@
       </c>
       <c r="M143" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N143" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N143" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12237,12 +12237,12 @@
       </c>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N144" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N144" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12301,12 +12301,12 @@
       </c>
       <c r="M145" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N145" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N145" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12365,12 +12365,12 @@
       </c>
       <c r="M146" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N146" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N146" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12429,12 +12429,12 @@
       </c>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N147" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N147" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12497,12 +12497,12 @@
       </c>
       <c r="M148" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N148" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N148" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>
@@ -12561,12 +12561,12 @@
       </c>
       <c r="M149" s="2" t="inlineStr">
         <is>
-          <t>not_deployed</t>
-        </is>
-      </c>
-      <c r="N149" s="2" t="inlineStr">
-        <is>
-          <t>ready to load through the Change Loader</t>
+          <t>bulk_upload</t>
+        </is>
+      </c>
+      <c r="N149" s="3" t="inlineStr">
+        <is>
+          <t>uploaded 2026-10-04, awaiting ID readback</t>
         </is>
       </c>
     </row>

</xml_diff>